<commit_message>
The tariff workbook: three sheets, the simple conversion on top and the values below; plot use and NAMA category tables added; the empty count explained
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/W16/analysis/meter_tariff_to_nama_category.xlsx
+++ b/W16/analysis/meter_tariff_to_nama_category.xlsx
@@ -7,8 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tariff to category" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Tariff" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Plot use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 NAMA category" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,30 +29,21 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="12"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
+    <font/>
     <font>
       <b val="1"/>
     </font>
     <font>
       <i val="1"/>
       <color rgb="00808080"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -88,36 +81,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -483,502 +471,826 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Electricity tariff  &gt;  NAMA demand category  &gt;  plot use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
           <t>Electricity tariff (as received)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NAMA water demand category</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Plot use it gives</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff (with National Subsidy)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Additional Account Tariff</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Residential-Commercial when the plot also carries domestic meters</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Fisheries</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Governmental</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>MOD</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Governmental</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural (irrigation pump)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural; Residential when a house is metered on the farm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Special consumption</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>CRT Seasonal; CRT Time of Use; CRT Fixed Rate</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>a consumption class (over 150 MWh/yr), not a use: each account resolved from public data, split below</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: shops, malls, fuel, banks, telecom, unresolved</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Commercial / Residential-Commercial</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: government, education, health, religious</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Governmental</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: industrial (Tanam estate)</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Special consumption</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: farm pumps (Al Aynayn)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>The same, with the values</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Electricity tariff (as received)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Meters</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>NAMA water demand category (PAM-GUD-201 s7.3)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Water rate applied</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Return to sewer</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Plot use it gives (land-use class)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Plot use it gives</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Primary Account Tariff</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B22" s="6" t="n">
         <v>10973</v>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Domestic</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>164 l/person/d x the settlement's persons per property (G201 Table 11, Adh Dhahirah)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>85 % (Table 19)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Residential: one property each</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>one property per meter</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Primary Account Tariff (with National Subsidy)</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B23" s="7" t="n">
         <v>5272</v>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Domestic</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>same</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>85 %</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Residential</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>one property per meter</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Additional Account Tariff</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B24" s="6" t="n">
         <v>6344</v>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Domestic</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>same</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>85 %</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Residential: a further property on the plot</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>a further property on the same plot</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B25" s="7" t="n">
         <v>9385</v>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Non-domestic</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>share of the 22 % of domestic (G201 Table 11, distributed ratio)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>54 % (Table 19)</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Commercial; Home and shop when the plot also carries a domestic meter</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Residential-Commercial when the plot also carries domestic meters</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>placed on the shop meters in proportion</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Fisheries</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B26" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Non-domestic</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>22 % share</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>Tourism</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B27" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Non-domestic</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>22 % share</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Commercial</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B28" s="6" t="n">
         <v>966</v>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Governmental</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>share of the 14 % of domestic (G201 Table 11, distributed ratio)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Government, when government meters outnumber shop and domestic meters on the plot</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>placed on the government meters in proportion</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>MOD</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B29" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Governmental</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>14 % share</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Agricultural</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B30" s="6" t="n">
         <v>523</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Agricultural (irrigation pump)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>none: no sewage</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Agricultural when farm meters only; Residential when a house is metered on the farm</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural; Residential when a house is metered on the farm</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>the farm carries no load, the house on it does</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Industrial</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B31" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Special consumption (identified project)</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Special consumption</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>93 l/worker/d, dry industry (G201 Table 12)</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Industrial</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>CRT Seasonal / CRT Time of Use / CRT Fixed Rate</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
+      <c r="G31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>CRT Seasonal; CRT Time of Use; CRT Fixed Rate</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
         <v>499</v>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>A consumption class (over 150 MWh/yr), not a use: each account resolved from public data, below</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr"/>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CRT found: Commercial, telecom/utility, unresolved</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="n">
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>a consumption class (over 150 MWh/yr), not a use: each account resolved from public data, split below</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>OpenStreetMap, reverse geocoding, satellite by eye, the identified-projects search</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: shops, malls, fuel, banks, telecom, unresolved</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
         <v>321</v>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Non-domestic</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>22 % share</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Commercial / Home and shop</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CRT found: Government, education, health, religious</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="n">
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Commercial / Residential-Commercial</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>110 unresolved accounts kept as non-domestic, flagged</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: government, education, health, religious</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
         <v>135</v>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Governmental</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>14 % share</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F34" s="3" t="inlineStr">
         <is>
           <t>Government</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CRT found: Industrial (Tanam estate)</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
+      <c r="G34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: industrial (Tanam estate)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Special consumption</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>93 l/worker/d</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>54 %</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Industrial</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   CRT found: Agricultural (Aynayn farm pumps)</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="n">
+      <c r="G35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   CRT found: farm pumps (Al Aynayn)</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Agricultural</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F36" s="3" t="inlineStr">
         <is>
           <t>Agricultural</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>All meters</t>
-        </is>
-      </c>
-      <c r="B17" s="9">
-        <f>SUM(B2:B12)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>(the four CRT lines are the split of the CRT line above them and are not summed)</t>
+      <c r="G36" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>The four CRT lines split the CRT line above them; the tariff lines sum to every meter.</t>
         </is>
       </c>
     </row>
@@ -993,82 +1305,954 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Plot use  &lt;  the meter types read as that use, and the other evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Plot use</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Meter types inferred as this use</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Other evidence (not a meter)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff; Primary Account Tariff (with National Subsidy); Additional Account Tariff</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Residential-Commercial</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>domestic tariffs with shop tariffs (Commercial, Fisheries, Tourism, CRT shops) on one plot</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Commercial; Fisheries; Tourism; CRT accounts found to be shops, malls, fuel, banks, telecom or unresolved</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Government; MOD; CRT accounts found to be government, education, health or religious</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>the treatment plant's compound (farm meters for its pumps), set by hand</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural; CRT accounts found to be farm pumps</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>planted, by satellite: green area of 1,000 m2 or more at NDVI 0.20, or 60 % green at NDVI 0.40 on a plot of 800 m2 or more</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Industrial; CRT accounts found to be industrial (Tanam estate); the estates' Commercial-tariff meters sit on these plots but do not decide the use</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>inside the Al Tayyeb or Tanam estate footprint (identified projects)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>none: no meter on these plots</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>the cadastre's Tourism class (the old quarters)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Empty (unmetered)</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>none: no meter of any tariff</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>not planted, not heritage, not in an estate; the cadastre's Proposed plots fall here when unmetered</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>The same, with the values</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Plot use</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Plots</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>of which with meters</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Meter types inferred as this use</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Other evidence (not a meter)</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Rule, in the order applied</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Load it carries</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Residential</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>12464</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>12464</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff; Primary Account Tariff (with National Subsidy); Additional Account Tariff</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>domestic meters are more than two-thirds of the plot's meters</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>domestic: persons per property x 164 l/d; the minority shop or government meters keep their share</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Residential-Commercial</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>614</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>614</v>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>domestic tariffs with shop tariffs (Commercial, Fisheries, Tourism, CRT shops) on one plot</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>no category reaches two-thirds and shop meters are at least as many as government meters</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>domestic and non-domestic, each on its own meters</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>1321</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1321</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Commercial; Fisheries; Tourism; CRT accounts found to be shops, malls, fuel, banks, telecom or unresolved</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>shop meters are two-thirds or more of the plot's meters</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>non-domestic: its share of the 22 %; any domestic meters on it keep theirs</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>410</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Government; MOD; CRT accounts found to be government, education, health or religious</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>the treatment plant's compound (farm meters for its pumps), set by hand</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>government meters are two-thirds or more; or a mix where government meters outnumber shop meters</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>governmental: its share of the 14 %; any domestic meters on it keep theirs</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>3398</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>1684</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Agricultural; CRT accounts found to be farm pumps</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>planted, by satellite: green area of 1,000 m2 or more at NDVI 0.20, or 60 % green at NDVI 0.40 on a plot of 800 m2 or more</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>a farm meter on the plot; or planted, unless the plot's meters are two-thirds shops or over half government</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>none for the farm; a house metered on it carries its domestic load</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>467</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>263</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Industrial; CRT accounts found to be industrial (Tanam estate); the estates' Commercial-tariff meters sit on these plots but do not decide the use</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>inside the Al Tayyeb or Tanam estate footprint (identified projects)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>inside an estate footprint; or special-consumption meters at least as many as domestic</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>special consumption: the estate's assumed workforce (4,500 and 1,800) spread by plot area at 93 l/worker/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Heritage</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>177</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>none: no meter on these plots</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>the cadastre's Tourism class (the old quarters)</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>the cadastre class is Tourism</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Empty (unmetered)</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>58414</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>none: no meter of any tariff</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>not planted, not heritage, not in an estate; the cadastre's Proposed plots fall here when unmetered</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>no meter and no other evidence</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>future people: home-shaped plots at 171.3 l/d per person as the settlement fills</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NAMA demand category  &lt;  the tariffs folded into it, and the plot uses that carry it</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>NAMA water demand category</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Electricity tariffs folded in</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Plot uses that carry its load</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff; Primary Account Tariff (with National Subsidy); Additional Account Tariff</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Residential; Residential-Commercial; the dwelling meters on farm, shop and government plots</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Fisheries; Tourism; CRT accounts found to be shops, malls, fuel, banks, telecom or unresolved</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Residential-Commercial; the shop meters on other plots</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Governmental</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Government; MOD; CRT accounts found to be government, education, health or religious</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Government; the government meters on other plots</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural; CRT accounts found to be farm pumps</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural (farm meters and planted plots)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Special consumption</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Industrial; CRT accounts found to be industrial (Tanam estate)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Industrial (the two estates' plots, by area)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>The same, with the values</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>NAMA water demand category</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Meters</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Electricity tariffs folded in</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Plot uses that carry its load</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Water rate</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Return to sewer</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Water 2024, m3/d</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Sewage 2024, m3/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Domestic</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>22589</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Primary Account Tariff; Primary Account Tariff (with National Subsidy); Additional Account Tariff</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Residential; Residential-Commercial; the dwelling meters on farm, shop and government plots</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>164 l/person/d x persons per property</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>85 %</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>19663</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>16713</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Non-domestic</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>9713</v>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Fisheries; Tourism; CRT accounts found to be shops, malls, fuel, banks, telecom or unresolved</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Commercial; Residential-Commercial; the shop meters on other plots</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>22 % of the settlement's domestic water, placed on its shop meters</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>54 %</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>4326</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>2336</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Governmental</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1102</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Government; MOD; CRT accounts found to be government, education, health or religious</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Government; the government meters on other plots</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>14 % of the settlement's domestic water, placed on its government meters</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>54 %</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>2753</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>551</v>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural; CRT accounts found to be farm pumps</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Agricultural (farm meters and planted plots)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>none: irrigation, no sewage</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Special consumption</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Industrial; CRT accounts found to be industrial (Tanam estate)</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Industrial (the two estates' plots, by area)</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>93 l/worker/d on the assumed workforce (4,500 Al Tayyeb, 1,800 Tanam)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>54 %</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>586</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>316</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="11" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Empty and Proposed</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Empty is a plot with no meter and no other evidence: 58,414 plots. The cadastre's Proposed class (49 plots) is not a use of its own: 38 are unmetered and count as empty, 11 carry meters and take their use from them. The report's figure of 60,509 empty plots is the cadastre's Future status, which also holds 1,714 planted plots, 177 heritage plots and 204 unbuilt estate plots; none of those carries future people.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Industrial estates</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Al Tayyeb and Tanam are metered as Commercial (1,035 and 409 meters). Their industrial plots are classed by the estate footprint and carry the special-consumption workforce (4,500 and 1,800 assumed), not the shop share.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Al Tayyeb and Tanam are metered as Commercial (1,035 and 409 meters). The estate footprint decides the use; the plots carry the assumed workforce, not the shop share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Heritage</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>The old quarters (177 plots) are classed from the cadastre, not the meters, and carry no load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Empty and Proposed plots</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>No meter: capacity for future people at 171.3 l/d each (164 x 0.85 + 36 x 0.54 + 23 x 0.54).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>The old quarters (177 plots) come from the cadastre's Tourism class, carry no meter and no load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Meters on no plot</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>126 meters lie more than 15 m from any plot and carry nothing until NWS says whether to assign or leave them (Design Basis Report, Section 3.3).</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Water and sewage 2024</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>The sums of the plot layer's 2024 water and sewage by category, m3/d, after the return ratios; the same figures the report's Table 6 builds on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>W14/shp/ELE_meters_on_plots.shp (33,971 accounts, 2024); rules in W14/py/plot_class_from_meters.py; categories per PAM-GUD-201 section 7.3; rates Table 11 (p60) and Table 19 (p71).</t>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>W14/shp/ELE_meters_on_plots.shp (33,971 accounts, 2024) and W14/shp/PLOTS_load.shp (77,265 plots) with the report's one override (the treatment plant's compound as Government); rules in W14/py/plot_class_v2_apply.py; categories per PAM-GUD-201 section 7.3; rates Table 11 (p60) and Table 19 (p71).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Property, not dwelling: the workbook's domestic line and the report's tariff footnote
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/W16/analysis/meter_tariff_to_nama_category.xlsx
+++ b/W16/analysis/meter_tariff_to_nama_category.xlsx
@@ -1846,7 +1846,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Residential; Residential-Commercial; the dwelling meters on farm, shop and government plots</t>
+          <t>Residential; Residential-Commercial; the domestic meters on farm, shop and government plots</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Residential; Residential-Commercial; the dwelling meters on farm, shop and government plots</t>
+          <t>Residential; Residential-Commercial; the domestic meters on farm, shop and government plots</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">

</xml_diff>